<commit_message>
NRI-0010: add era-aware dates with shared era key, per-entity BC flags, popup and import support, additive migration with backup and key backfill, sync specs and archive change
</commit_message>
<xml_diff>
--- a/resources/import_template.xlsx
+++ b/resources/import_template.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,6 +562,28 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>Поляна</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Заговор</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>15 марта 44 г. до н.э.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-0043-03-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Сговор против Цезаря</t>
         </is>
       </c>
     </row>

</xml_diff>